<commit_message>
v3.0.0: aplicación de escritorio instalable
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/storage/templates/Bar_Piscina.xlsx
+++ b/storage/templates/Bar_Piscina.xlsx
@@ -709,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AN1005"/>
+  <dimension ref="A1:AN1017"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="10.77734375" customWidth="1" style="1" min="1" max="1"/>
@@ -7927,78 +7927,882 @@
         <v/>
       </c>
     </row>
-    <row r="108" ht="22.05" customHeight="1">
-      <c r="C108" s="11">
-        <f>SUM(C7:C107)</f>
-        <v/>
-      </c>
-      <c r="D108" s="12" t="n"/>
-      <c r="E108" s="13" t="inlineStr">
+    <row r="108" ht="25.05" customHeight="1">
+      <c r="A108" s="27" t="inlineStr">
+        <is>
+          <t>2715</t>
+        </is>
+      </c>
+      <c r="B108" s="27" t="inlineStr">
+        <is>
+          <t>CONO HELADO 45 MM</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D108" s="33" t="inlineStr">
+        <is>
+          <t>UNIDAD</t>
+        </is>
+      </c>
+      <c r="E108" s="9" t="n">
+        <v>0.16584</v>
+      </c>
+      <c r="F108" s="10">
+        <f>C108*E108</f>
+        <v/>
+      </c>
+      <c r="G108" s="22" t="n"/>
+      <c r="H108" s="22" t="n"/>
+      <c r="I108" s="22" t="n"/>
+      <c r="J108" s="22" t="n"/>
+      <c r="K108" s="22" t="n"/>
+      <c r="L108" s="22" t="n"/>
+      <c r="M108" s="22" t="n"/>
+      <c r="N108" s="22" t="n"/>
+      <c r="O108" s="22" t="n"/>
+      <c r="P108" s="22" t="n"/>
+      <c r="Q108" s="22" t="n"/>
+      <c r="R108" s="22" t="n"/>
+      <c r="S108" s="22" t="n"/>
+      <c r="T108" s="22" t="n"/>
+      <c r="U108" s="22" t="n"/>
+      <c r="V108" s="22" t="n"/>
+      <c r="W108" s="22" t="n"/>
+      <c r="X108" s="22" t="n"/>
+      <c r="Y108" s="22" t="n"/>
+      <c r="Z108" s="22" t="n"/>
+      <c r="AA108" s="22" t="n"/>
+      <c r="AB108" s="22" t="n"/>
+      <c r="AC108" s="22" t="n"/>
+      <c r="AD108" s="22" t="n"/>
+      <c r="AE108" s="22" t="n"/>
+      <c r="AF108" s="22" t="n"/>
+      <c r="AG108" s="22" t="n"/>
+      <c r="AH108" s="22" t="n"/>
+      <c r="AI108" s="22" t="n"/>
+      <c r="AJ108" s="22" t="n"/>
+      <c r="AK108" s="22" t="n"/>
+      <c r="AL108" s="23">
+        <f>SUM(G108:AK108)</f>
+        <v/>
+      </c>
+      <c r="AM108" s="24">
+        <f>SUM(C108,AL108)</f>
+        <v/>
+      </c>
+      <c r="AN108" s="25">
+        <f>E108*AM108</f>
+        <v/>
+      </c>
+    </row>
+    <row r="109" ht="25.05" customHeight="1">
+      <c r="A109" s="27" t="inlineStr">
+        <is>
+          <t>17116</t>
+        </is>
+      </c>
+      <c r="B109" s="27" t="inlineStr">
+        <is>
+          <t>HELADO GRANEL PREMIUM VAINILLA</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D109" s="33" t="inlineStr">
+        <is>
+          <t>LITRO</t>
+        </is>
+      </c>
+      <c r="E109" s="9" t="n">
+        <v>3.82304</v>
+      </c>
+      <c r="F109" s="10">
+        <f>C109*E109</f>
+        <v/>
+      </c>
+      <c r="G109" s="22" t="n"/>
+      <c r="H109" s="22" t="n"/>
+      <c r="I109" s="22" t="n"/>
+      <c r="J109" s="22" t="n"/>
+      <c r="K109" s="22" t="n"/>
+      <c r="L109" s="22" t="n"/>
+      <c r="M109" s="22" t="n"/>
+      <c r="N109" s="22" t="n"/>
+      <c r="O109" s="22" t="n"/>
+      <c r="P109" s="22" t="n"/>
+      <c r="Q109" s="22" t="n"/>
+      <c r="R109" s="22" t="n"/>
+      <c r="S109" s="22" t="n"/>
+      <c r="T109" s="22" t="n"/>
+      <c r="U109" s="22" t="n"/>
+      <c r="V109" s="22" t="n"/>
+      <c r="W109" s="22" t="n"/>
+      <c r="X109" s="22" t="n"/>
+      <c r="Y109" s="22" t="n"/>
+      <c r="Z109" s="22" t="n"/>
+      <c r="AA109" s="22" t="n"/>
+      <c r="AB109" s="22" t="n"/>
+      <c r="AC109" s="22" t="n"/>
+      <c r="AD109" s="22" t="n"/>
+      <c r="AE109" s="22" t="n"/>
+      <c r="AF109" s="22" t="n"/>
+      <c r="AG109" s="22" t="n"/>
+      <c r="AH109" s="22" t="n"/>
+      <c r="AI109" s="22" t="n"/>
+      <c r="AJ109" s="22" t="n"/>
+      <c r="AK109" s="22" t="n"/>
+      <c r="AL109" s="23">
+        <f>SUM(G109:AK109)</f>
+        <v/>
+      </c>
+      <c r="AM109" s="24">
+        <f>SUM(C109,AL109)</f>
+        <v/>
+      </c>
+      <c r="AN109" s="25">
+        <f>E109*AM109</f>
+        <v/>
+      </c>
+    </row>
+    <row r="110" ht="25.05" customHeight="1">
+      <c r="A110" s="27" t="inlineStr">
+        <is>
+          <t>22213</t>
+        </is>
+      </c>
+      <c r="B110" s="27" t="inlineStr">
+        <is>
+          <t>HELADO GRANEL ESPECIAL TURRON</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D110" s="33" t="inlineStr">
+        <is>
+          <t>LITRO</t>
+        </is>
+      </c>
+      <c r="E110" s="9" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="F110" s="10">
+        <f>C110*E110</f>
+        <v/>
+      </c>
+      <c r="G110" s="22" t="n"/>
+      <c r="H110" s="22" t="n"/>
+      <c r="I110" s="22" t="n"/>
+      <c r="J110" s="22" t="n"/>
+      <c r="K110" s="22" t="n"/>
+      <c r="L110" s="22" t="n"/>
+      <c r="M110" s="22" t="n"/>
+      <c r="N110" s="22" t="n"/>
+      <c r="O110" s="22" t="n"/>
+      <c r="P110" s="22" t="n"/>
+      <c r="Q110" s="22" t="n"/>
+      <c r="R110" s="22" t="n"/>
+      <c r="S110" s="22" t="n"/>
+      <c r="T110" s="22" t="n"/>
+      <c r="U110" s="22" t="n"/>
+      <c r="V110" s="22" t="n"/>
+      <c r="W110" s="22" t="n"/>
+      <c r="X110" s="22" t="n"/>
+      <c r="Y110" s="22" t="n"/>
+      <c r="Z110" s="22" t="n"/>
+      <c r="AA110" s="22" t="n"/>
+      <c r="AB110" s="22" t="n"/>
+      <c r="AC110" s="22" t="n"/>
+      <c r="AD110" s="22" t="n"/>
+      <c r="AE110" s="22" t="n"/>
+      <c r="AF110" s="22" t="n"/>
+      <c r="AG110" s="22" t="n"/>
+      <c r="AH110" s="22" t="n"/>
+      <c r="AI110" s="22" t="n"/>
+      <c r="AJ110" s="22" t="n"/>
+      <c r="AK110" s="22" t="n"/>
+      <c r="AL110" s="23">
+        <f>SUM(G110:AK110)</f>
+        <v/>
+      </c>
+      <c r="AM110" s="24">
+        <f>SUM(C110,AL110)</f>
+        <v/>
+      </c>
+      <c r="AN110" s="25">
+        <f>E110*AM110</f>
+        <v/>
+      </c>
+    </row>
+    <row r="111" ht="25.05" customHeight="1">
+      <c r="A111" s="27" t="inlineStr">
+        <is>
+          <t>22218</t>
+        </is>
+      </c>
+      <c r="B111" s="27" t="inlineStr">
+        <is>
+          <t>HELADO GRANEL ESPECIAL GALLETA MARIA</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D111" s="33" t="inlineStr">
+        <is>
+          <t>LITRO</t>
+        </is>
+      </c>
+      <c r="E111" s="9" t="n">
+        <v>5.09271</v>
+      </c>
+      <c r="F111" s="10">
+        <f>C111*E111</f>
+        <v/>
+      </c>
+      <c r="G111" s="22" t="n"/>
+      <c r="H111" s="22" t="n"/>
+      <c r="I111" s="22" t="n"/>
+      <c r="J111" s="22" t="n"/>
+      <c r="K111" s="22" t="n"/>
+      <c r="L111" s="22" t="n"/>
+      <c r="M111" s="22" t="n"/>
+      <c r="N111" s="22" t="n"/>
+      <c r="O111" s="22" t="n"/>
+      <c r="P111" s="22" t="n"/>
+      <c r="Q111" s="22" t="n"/>
+      <c r="R111" s="22" t="n"/>
+      <c r="S111" s="22" t="n"/>
+      <c r="T111" s="22" t="n"/>
+      <c r="U111" s="22" t="n"/>
+      <c r="V111" s="22" t="n"/>
+      <c r="W111" s="22" t="n"/>
+      <c r="X111" s="22" t="n"/>
+      <c r="Y111" s="22" t="n"/>
+      <c r="Z111" s="22" t="n"/>
+      <c r="AA111" s="22" t="n"/>
+      <c r="AB111" s="22" t="n"/>
+      <c r="AC111" s="22" t="n"/>
+      <c r="AD111" s="22" t="n"/>
+      <c r="AE111" s="22" t="n"/>
+      <c r="AF111" s="22" t="n"/>
+      <c r="AG111" s="22" t="n"/>
+      <c r="AH111" s="22" t="n"/>
+      <c r="AI111" s="22" t="n"/>
+      <c r="AJ111" s="22" t="n"/>
+      <c r="AK111" s="22" t="n"/>
+      <c r="AL111" s="23">
+        <f>SUM(G111:AK111)</f>
+        <v/>
+      </c>
+      <c r="AM111" s="24">
+        <f>SUM(C111,AL111)</f>
+        <v/>
+      </c>
+      <c r="AN111" s="25">
+        <f>E111*AM111</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112" ht="25.05" customHeight="1">
+      <c r="A112" s="27" t="inlineStr">
+        <is>
+          <t>22219</t>
+        </is>
+      </c>
+      <c r="B112" s="27" t="inlineStr">
+        <is>
+          <t>HELADO GRANEL ESPECIAL PISTACHO</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D112" s="33" t="inlineStr">
+        <is>
+          <t>LITRO</t>
+        </is>
+      </c>
+      <c r="E112" s="9" t="n">
+        <v>5.10031</v>
+      </c>
+      <c r="F112" s="10">
+        <f>C112*E112</f>
+        <v/>
+      </c>
+      <c r="G112" s="22" t="n"/>
+      <c r="H112" s="22" t="n"/>
+      <c r="I112" s="22" t="n"/>
+      <c r="J112" s="22" t="n"/>
+      <c r="K112" s="22" t="n"/>
+      <c r="L112" s="22" t="n"/>
+      <c r="M112" s="22" t="n"/>
+      <c r="N112" s="22" t="n"/>
+      <c r="O112" s="22" t="n"/>
+      <c r="P112" s="22" t="n"/>
+      <c r="Q112" s="22" t="n"/>
+      <c r="R112" s="22" t="n"/>
+      <c r="S112" s="22" t="n"/>
+      <c r="T112" s="22" t="n"/>
+      <c r="U112" s="22" t="n"/>
+      <c r="V112" s="22" t="n"/>
+      <c r="W112" s="22" t="n"/>
+      <c r="X112" s="22" t="n"/>
+      <c r="Y112" s="22" t="n"/>
+      <c r="Z112" s="22" t="n"/>
+      <c r="AA112" s="22" t="n"/>
+      <c r="AB112" s="22" t="n"/>
+      <c r="AC112" s="22" t="n"/>
+      <c r="AD112" s="22" t="n"/>
+      <c r="AE112" s="22" t="n"/>
+      <c r="AF112" s="22" t="n"/>
+      <c r="AG112" s="22" t="n"/>
+      <c r="AH112" s="22" t="n"/>
+      <c r="AI112" s="22" t="n"/>
+      <c r="AJ112" s="22" t="n"/>
+      <c r="AK112" s="22" t="n"/>
+      <c r="AL112" s="23">
+        <f>SUM(G112:AK112)</f>
+        <v/>
+      </c>
+      <c r="AM112" s="24">
+        <f>SUM(C112,AL112)</f>
+        <v/>
+      </c>
+      <c r="AN112" s="25">
+        <f>E112*AM112</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113" ht="25.05" customHeight="1">
+      <c r="A113" s="27" t="inlineStr">
+        <is>
+          <t>22245</t>
+        </is>
+      </c>
+      <c r="B113" s="27" t="inlineStr">
+        <is>
+          <t>HELADO GRANEL ESPECIAL CHEESECAKE</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D113" s="33" t="inlineStr">
+        <is>
+          <t>LITRO</t>
+        </is>
+      </c>
+      <c r="E113" s="9" t="n">
+        <v>4.58173</v>
+      </c>
+      <c r="F113" s="10">
+        <f>C113*E113</f>
+        <v/>
+      </c>
+      <c r="G113" s="22" t="n"/>
+      <c r="H113" s="22" t="n"/>
+      <c r="I113" s="22" t="n"/>
+      <c r="J113" s="22" t="n"/>
+      <c r="K113" s="22" t="n"/>
+      <c r="L113" s="22" t="n"/>
+      <c r="M113" s="22" t="n"/>
+      <c r="N113" s="22" t="n"/>
+      <c r="O113" s="22" t="n"/>
+      <c r="P113" s="22" t="n"/>
+      <c r="Q113" s="22" t="n"/>
+      <c r="R113" s="22" t="n"/>
+      <c r="S113" s="22" t="n"/>
+      <c r="T113" s="22" t="n"/>
+      <c r="U113" s="22" t="n"/>
+      <c r="V113" s="22" t="n"/>
+      <c r="W113" s="22" t="n"/>
+      <c r="X113" s="22" t="n"/>
+      <c r="Y113" s="22" t="n"/>
+      <c r="Z113" s="22" t="n"/>
+      <c r="AA113" s="22" t="n"/>
+      <c r="AB113" s="22" t="n"/>
+      <c r="AC113" s="22" t="n"/>
+      <c r="AD113" s="22" t="n"/>
+      <c r="AE113" s="22" t="n"/>
+      <c r="AF113" s="22" t="n"/>
+      <c r="AG113" s="22" t="n"/>
+      <c r="AH113" s="22" t="n"/>
+      <c r="AI113" s="22" t="n"/>
+      <c r="AJ113" s="22" t="n"/>
+      <c r="AK113" s="22" t="n"/>
+      <c r="AL113" s="23">
+        <f>SUM(G113:AK113)</f>
+        <v/>
+      </c>
+      <c r="AM113" s="24">
+        <f>SUM(C113,AL113)</f>
+        <v/>
+      </c>
+      <c r="AN113" s="25">
+        <f>E113*AM113</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114" ht="25.05" customHeight="1">
+      <c r="A114" s="27" t="inlineStr">
+        <is>
+          <t>22246</t>
+        </is>
+      </c>
+      <c r="B114" s="27" t="inlineStr">
+        <is>
+          <t>HELADO GRANEL ESPECIAL KIT-KAT</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D114" s="33" t="inlineStr">
+        <is>
+          <t>LITRO</t>
+        </is>
+      </c>
+      <c r="E114" s="9" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F114" s="10">
+        <f>C114*E114</f>
+        <v/>
+      </c>
+      <c r="G114" s="22" t="n"/>
+      <c r="H114" s="22" t="n"/>
+      <c r="I114" s="22" t="n"/>
+      <c r="J114" s="22" t="n"/>
+      <c r="K114" s="22" t="n"/>
+      <c r="L114" s="22" t="n"/>
+      <c r="M114" s="22" t="n"/>
+      <c r="N114" s="22" t="n"/>
+      <c r="O114" s="22" t="n"/>
+      <c r="P114" s="22" t="n"/>
+      <c r="Q114" s="22" t="n"/>
+      <c r="R114" s="22" t="n"/>
+      <c r="S114" s="22" t="n"/>
+      <c r="T114" s="22" t="n"/>
+      <c r="U114" s="22" t="n"/>
+      <c r="V114" s="22" t="n"/>
+      <c r="W114" s="22" t="n"/>
+      <c r="X114" s="22" t="n"/>
+      <c r="Y114" s="22" t="n"/>
+      <c r="Z114" s="22" t="n"/>
+      <c r="AA114" s="22" t="n"/>
+      <c r="AB114" s="22" t="n"/>
+      <c r="AC114" s="22" t="n"/>
+      <c r="AD114" s="22" t="n"/>
+      <c r="AE114" s="22" t="n"/>
+      <c r="AF114" s="22" t="n"/>
+      <c r="AG114" s="22" t="n"/>
+      <c r="AH114" s="22" t="n"/>
+      <c r="AI114" s="22" t="n"/>
+      <c r="AJ114" s="22" t="n"/>
+      <c r="AK114" s="22" t="n"/>
+      <c r="AL114" s="23">
+        <f>SUM(G114:AK114)</f>
+        <v/>
+      </c>
+      <c r="AM114" s="24">
+        <f>SUM(C114,AL114)</f>
+        <v/>
+      </c>
+      <c r="AN114" s="25">
+        <f>E114*AM114</f>
+        <v/>
+      </c>
+    </row>
+    <row r="115" ht="25.05" customHeight="1">
+      <c r="A115" s="27" t="inlineStr">
+        <is>
+          <t>22251</t>
+        </is>
+      </c>
+      <c r="B115" s="27" t="inlineStr">
+        <is>
+          <t>HELADO GRANEL ESPECIAL DULCE DE LECHE</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D115" s="33" t="inlineStr">
+        <is>
+          <t>LITRO</t>
+        </is>
+      </c>
+      <c r="E115" s="9" t="n">
+        <v>4.58173</v>
+      </c>
+      <c r="F115" s="10">
+        <f>C115*E115</f>
+        <v/>
+      </c>
+      <c r="G115" s="22" t="n"/>
+      <c r="H115" s="22" t="n"/>
+      <c r="I115" s="22" t="n"/>
+      <c r="J115" s="22" t="n"/>
+      <c r="K115" s="22" t="n"/>
+      <c r="L115" s="22" t="n"/>
+      <c r="M115" s="22" t="n"/>
+      <c r="N115" s="22" t="n"/>
+      <c r="O115" s="22" t="n"/>
+      <c r="P115" s="22" t="n"/>
+      <c r="Q115" s="22" t="n"/>
+      <c r="R115" s="22" t="n"/>
+      <c r="S115" s="22" t="n"/>
+      <c r="T115" s="22" t="n"/>
+      <c r="U115" s="22" t="n"/>
+      <c r="V115" s="22" t="n"/>
+      <c r="W115" s="22" t="n"/>
+      <c r="X115" s="22" t="n"/>
+      <c r="Y115" s="22" t="n"/>
+      <c r="Z115" s="22" t="n"/>
+      <c r="AA115" s="22" t="n"/>
+      <c r="AB115" s="22" t="n"/>
+      <c r="AC115" s="22" t="n"/>
+      <c r="AD115" s="22" t="n"/>
+      <c r="AE115" s="22" t="n"/>
+      <c r="AF115" s="22" t="n"/>
+      <c r="AG115" s="22" t="n"/>
+      <c r="AH115" s="22" t="n"/>
+      <c r="AI115" s="22" t="n"/>
+      <c r="AJ115" s="22" t="n"/>
+      <c r="AK115" s="22" t="n"/>
+      <c r="AL115" s="23">
+        <f>SUM(G115:AK115)</f>
+        <v/>
+      </c>
+      <c r="AM115" s="24">
+        <f>SUM(C115,AL115)</f>
+        <v/>
+      </c>
+      <c r="AN115" s="25">
+        <f>E115*AM115</f>
+        <v/>
+      </c>
+    </row>
+    <row r="116" ht="25.05" customHeight="1">
+      <c r="A116" s="27" t="inlineStr">
+        <is>
+          <t>23557</t>
+        </is>
+      </c>
+      <c r="B116" s="27" t="inlineStr">
+        <is>
+          <t>HELADO GRANEL ESPECIAL NATA C/NUECES</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D116" s="33" t="inlineStr">
+        <is>
+          <t>LITRO</t>
+        </is>
+      </c>
+      <c r="E116" s="9" t="n">
+        <v>5.09271</v>
+      </c>
+      <c r="F116" s="10">
+        <f>C116*E116</f>
+        <v/>
+      </c>
+      <c r="G116" s="22" t="n"/>
+      <c r="H116" s="22" t="n"/>
+      <c r="I116" s="22" t="n"/>
+      <c r="J116" s="22" t="n"/>
+      <c r="K116" s="22" t="n"/>
+      <c r="L116" s="22" t="n"/>
+      <c r="M116" s="22" t="n"/>
+      <c r="N116" s="22" t="n"/>
+      <c r="O116" s="22" t="n"/>
+      <c r="P116" s="22" t="n"/>
+      <c r="Q116" s="22" t="n"/>
+      <c r="R116" s="22" t="n"/>
+      <c r="S116" s="22" t="n"/>
+      <c r="T116" s="22" t="n"/>
+      <c r="U116" s="22" t="n"/>
+      <c r="V116" s="22" t="n"/>
+      <c r="W116" s="22" t="n"/>
+      <c r="X116" s="22" t="n"/>
+      <c r="Y116" s="22" t="n"/>
+      <c r="Z116" s="22" t="n"/>
+      <c r="AA116" s="22" t="n"/>
+      <c r="AB116" s="22" t="n"/>
+      <c r="AC116" s="22" t="n"/>
+      <c r="AD116" s="22" t="n"/>
+      <c r="AE116" s="22" t="n"/>
+      <c r="AF116" s="22" t="n"/>
+      <c r="AG116" s="22" t="n"/>
+      <c r="AH116" s="22" t="n"/>
+      <c r="AI116" s="22" t="n"/>
+      <c r="AJ116" s="22" t="n"/>
+      <c r="AK116" s="22" t="n"/>
+      <c r="AL116" s="23">
+        <f>SUM(G116:AK116)</f>
+        <v/>
+      </c>
+      <c r="AM116" s="24">
+        <f>SUM(C116,AL116)</f>
+        <v/>
+      </c>
+      <c r="AN116" s="25">
+        <f>E116*AM116</f>
+        <v/>
+      </c>
+    </row>
+    <row r="117" ht="25.05" customHeight="1">
+      <c r="A117" s="27" t="inlineStr">
+        <is>
+          <t>700514</t>
+        </is>
+      </c>
+      <c r="B117" s="27" t="inlineStr">
+        <is>
+          <t>HELADO GRANEL CHOCOLATE</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D117" s="33" t="inlineStr">
+        <is>
+          <t>LITRO</t>
+        </is>
+      </c>
+      <c r="E117" s="9" t="n">
+        <v>1.2058</v>
+      </c>
+      <c r="F117" s="10">
+        <f>C117*E117</f>
+        <v/>
+      </c>
+      <c r="G117" s="22" t="n"/>
+      <c r="H117" s="22" t="n"/>
+      <c r="I117" s="22" t="n"/>
+      <c r="J117" s="22" t="n"/>
+      <c r="K117" s="22" t="n"/>
+      <c r="L117" s="22" t="n"/>
+      <c r="M117" s="22" t="n"/>
+      <c r="N117" s="22" t="n"/>
+      <c r="O117" s="22" t="n"/>
+      <c r="P117" s="22" t="n"/>
+      <c r="Q117" s="22" t="n"/>
+      <c r="R117" s="22" t="n"/>
+      <c r="S117" s="22" t="n"/>
+      <c r="T117" s="22" t="n"/>
+      <c r="U117" s="22" t="n"/>
+      <c r="V117" s="22" t="n"/>
+      <c r="W117" s="22" t="n"/>
+      <c r="X117" s="22" t="n"/>
+      <c r="Y117" s="22" t="n"/>
+      <c r="Z117" s="22" t="n"/>
+      <c r="AA117" s="22" t="n"/>
+      <c r="AB117" s="22" t="n"/>
+      <c r="AC117" s="22" t="n"/>
+      <c r="AD117" s="22" t="n"/>
+      <c r="AE117" s="22" t="n"/>
+      <c r="AF117" s="22" t="n"/>
+      <c r="AG117" s="22" t="n"/>
+      <c r="AH117" s="22" t="n"/>
+      <c r="AI117" s="22" t="n"/>
+      <c r="AJ117" s="22" t="n"/>
+      <c r="AK117" s="22" t="n"/>
+      <c r="AL117" s="23">
+        <f>SUM(G117:AK117)</f>
+        <v/>
+      </c>
+      <c r="AM117" s="24">
+        <f>SUM(C117,AL117)</f>
+        <v/>
+      </c>
+      <c r="AN117" s="25">
+        <f>E117*AM117</f>
+        <v/>
+      </c>
+    </row>
+    <row r="118" ht="25.05" customHeight="1">
+      <c r="A118" s="27" t="inlineStr">
+        <is>
+          <t>11207</t>
+        </is>
+      </c>
+      <c r="B118" s="27" t="inlineStr">
+        <is>
+          <t>HEL NESTLE BISCUIT AL CARAMELO 12 UDS</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D118" s="33" t="inlineStr">
+        <is>
+          <t>UNIDAD</t>
+        </is>
+      </c>
+      <c r="E118" s="9" t="n">
+        <v>1.37452</v>
+      </c>
+      <c r="F118" s="10">
+        <f>C118*E118</f>
+        <v/>
+      </c>
+      <c r="G118" s="22" t="n"/>
+      <c r="H118" s="22" t="n"/>
+      <c r="I118" s="22" t="n"/>
+      <c r="J118" s="22" t="n"/>
+      <c r="K118" s="22" t="n"/>
+      <c r="L118" s="22" t="n"/>
+      <c r="M118" s="22" t="n"/>
+      <c r="N118" s="22" t="n"/>
+      <c r="O118" s="22" t="n"/>
+      <c r="P118" s="22" t="n"/>
+      <c r="Q118" s="22" t="n"/>
+      <c r="R118" s="22" t="n"/>
+      <c r="S118" s="22" t="n"/>
+      <c r="T118" s="22" t="n"/>
+      <c r="U118" s="22" t="n"/>
+      <c r="V118" s="22" t="n"/>
+      <c r="W118" s="22" t="n"/>
+      <c r="X118" s="22" t="n"/>
+      <c r="Y118" s="22" t="n"/>
+      <c r="Z118" s="22" t="n"/>
+      <c r="AA118" s="22" t="n"/>
+      <c r="AB118" s="22" t="n"/>
+      <c r="AC118" s="22" t="n"/>
+      <c r="AD118" s="22" t="n"/>
+      <c r="AE118" s="22" t="n"/>
+      <c r="AF118" s="22" t="n"/>
+      <c r="AG118" s="22" t="n"/>
+      <c r="AH118" s="22" t="n"/>
+      <c r="AI118" s="22" t="n"/>
+      <c r="AJ118" s="22" t="n"/>
+      <c r="AK118" s="22" t="n"/>
+      <c r="AL118" s="23">
+        <f>SUM(G118:AK118)</f>
+        <v/>
+      </c>
+      <c r="AM118" s="24">
+        <f>SUM(C118,AL118)</f>
+        <v/>
+      </c>
+      <c r="AN118" s="25">
+        <f>E118*AM118</f>
+        <v/>
+      </c>
+    </row>
+    <row r="119" ht="25.05" customHeight="1">
+      <c r="A119" s="27" t="inlineStr">
+        <is>
+          <t>10121</t>
+        </is>
+      </c>
+      <c r="B119" s="27" t="inlineStr">
+        <is>
+          <t>CAVA PINKY S/ALCOHOL 75 CL (NIÑOS)</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D119" s="33" t="inlineStr">
+        <is>
+          <t>BOTELLA</t>
+        </is>
+      </c>
+      <c r="E119" s="9" t="n">
+        <v>4.32907</v>
+      </c>
+      <c r="F119" s="10">
+        <f>C119*E119</f>
+        <v/>
+      </c>
+      <c r="G119" s="22" t="n"/>
+      <c r="H119" s="22" t="n"/>
+      <c r="I119" s="22" t="n"/>
+      <c r="J119" s="22" t="n"/>
+      <c r="K119" s="22" t="n"/>
+      <c r="L119" s="22" t="n"/>
+      <c r="M119" s="22" t="n"/>
+      <c r="N119" s="22" t="n"/>
+      <c r="O119" s="22" t="n"/>
+      <c r="P119" s="22" t="n"/>
+      <c r="Q119" s="22" t="n"/>
+      <c r="R119" s="22" t="n"/>
+      <c r="S119" s="22" t="n"/>
+      <c r="T119" s="22" t="n"/>
+      <c r="U119" s="22" t="n"/>
+      <c r="V119" s="22" t="n"/>
+      <c r="W119" s="22" t="n"/>
+      <c r="X119" s="22" t="n"/>
+      <c r="Y119" s="22" t="n"/>
+      <c r="Z119" s="22" t="n"/>
+      <c r="AA119" s="22" t="n"/>
+      <c r="AB119" s="22" t="n"/>
+      <c r="AC119" s="22" t="n"/>
+      <c r="AD119" s="22" t="n"/>
+      <c r="AE119" s="22" t="n"/>
+      <c r="AF119" s="22" t="n"/>
+      <c r="AG119" s="22" t="n"/>
+      <c r="AH119" s="22" t="n"/>
+      <c r="AI119" s="22" t="n"/>
+      <c r="AJ119" s="22" t="n"/>
+      <c r="AK119" s="22" t="n"/>
+      <c r="AL119" s="23">
+        <f>SUM(G119:AK119)</f>
+        <v/>
+      </c>
+      <c r="AM119" s="24">
+        <f>SUM(C119,AL119)</f>
+        <v/>
+      </c>
+      <c r="AN119" s="25">
+        <f>E119*AM119</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120" ht="22.05" customHeight="1">
+      <c r="C120" s="11">
+        <f>SUM(C7:C119)</f>
+        <v/>
+      </c>
+      <c r="D120" s="12" t="n"/>
+      <c r="E120" s="13" t="inlineStr">
         <is>
           <t>ESTOCAJE  INICIAL</t>
         </is>
       </c>
-      <c r="F108" s="14">
-        <f>SUM(F7:F107)</f>
-        <v/>
-      </c>
-      <c r="AL108" s="11">
-        <f>SUM(AL7:AL107)</f>
-        <v/>
-      </c>
-      <c r="AM108" s="24">
-        <f>SUM(AM7:AM107)</f>
-        <v/>
-      </c>
-      <c r="AN108" s="26">
-        <f>SUM(AN7:AN107)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="109" ht="22.05" customHeight="1">
-      <c r="E109" s="3" t="n"/>
-      <c r="F109" s="3" t="n"/>
-      <c r="AN109" s="21" t="n"/>
-    </row>
-    <row r="110" ht="22.05" customHeight="1">
-      <c r="E110" s="3" t="n"/>
-      <c r="F110" s="3" t="n"/>
-      <c r="AN110" s="21" t="n"/>
-    </row>
-    <row r="111" ht="22.05" customHeight="1">
-      <c r="AN111" s="21" t="n"/>
-    </row>
-    <row r="112" ht="22.05" customHeight="1">
-      <c r="AN112" s="21" t="n"/>
-    </row>
-    <row r="113" ht="22.05" customHeight="1">
-      <c r="AN113" s="21" t="n"/>
-    </row>
-    <row r="114" ht="22.05" customHeight="1">
-      <c r="AN114" s="21" t="n"/>
-    </row>
-    <row r="115" ht="22.05" customHeight="1">
-      <c r="AN115" s="21" t="n"/>
-    </row>
-    <row r="116" ht="22.05" customHeight="1">
-      <c r="AN116" s="21" t="n"/>
-    </row>
-    <row r="117" ht="22.05" customHeight="1">
-      <c r="AN117" s="21" t="n"/>
-    </row>
-    <row r="118" ht="22.05" customHeight="1">
-      <c r="AN118" s="21" t="n"/>
-    </row>
-    <row r="119" ht="22.05" customHeight="1">
-      <c r="AN119" s="21" t="n"/>
-    </row>
-    <row r="120" ht="22.05" customHeight="1">
-      <c r="AN120" s="21" t="n"/>
+      <c r="F120" s="14">
+        <f>SUM(F7:F119)</f>
+        <v/>
+      </c>
+      <c r="AL120" s="11">
+        <f>SUM(AL7:AL119)</f>
+        <v/>
+      </c>
+      <c r="AM120" s="24">
+        <f>SUM(AM7:AM119)</f>
+        <v/>
+      </c>
+      <c r="AN120" s="26">
+        <f>SUM(AN7:AN119)</f>
+        <v/>
+      </c>
     </row>
     <row r="121" ht="22.05" customHeight="1">
+      <c r="E121" s="3" t="n"/>
+      <c r="F121" s="3" t="n"/>
       <c r="AN121" s="21" t="n"/>
     </row>
     <row r="122" ht="22.05" customHeight="1">
+      <c r="E122" s="3" t="n"/>
+      <c r="F122" s="3" t="n"/>
       <c r="AN122" s="21" t="n"/>
     </row>
     <row r="123" ht="22.05" customHeight="1">
@@ -10649,6 +11453,42 @@
     </row>
     <row r="1005">
       <c r="AN1005" s="21" t="n"/>
+    </row>
+    <row r="1006">
+      <c r="AN1006" s="21" t="n"/>
+    </row>
+    <row r="1007">
+      <c r="AN1007" s="21" t="n"/>
+    </row>
+    <row r="1008">
+      <c r="AN1008" s="21" t="n"/>
+    </row>
+    <row r="1009">
+      <c r="AN1009" s="21" t="n"/>
+    </row>
+    <row r="1010">
+      <c r="AN1010" s="21" t="n"/>
+    </row>
+    <row r="1011">
+      <c r="AN1011" s="21" t="n"/>
+    </row>
+    <row r="1012">
+      <c r="AN1012" s="21" t="n"/>
+    </row>
+    <row r="1013">
+      <c r="AN1013" s="21" t="n"/>
+    </row>
+    <row r="1014">
+      <c r="AN1014" s="21" t="n"/>
+    </row>
+    <row r="1015">
+      <c r="AN1015" s="21" t="n"/>
+    </row>
+    <row r="1016">
+      <c r="AN1016" s="21" t="n"/>
+    </row>
+    <row r="1017">
+      <c r="AN1017" s="21" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A6:F6"/>

</xml_diff>